<commit_message>
Pantallas del Sprint 1, estimación del equipo y entregables actualizados
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtGmXDVgEBa1Hp6paBTjbG
</commit_message>
<xml_diff>
--- a/entregables/SIGRO - Plan de los dos sprints.xlsx
+++ b/entregables/SIGRO - Plan de los dos sprints.xlsx
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="F37" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Total: 152 puntos en 29 historias.  Reparto: Fernando Istaña 21 · Henry Ticona 63 · Nicolás Pachamora 31 · Víctor Luján 37</t>
+          <t>Total: 153 puntos en 29 historias.  Reparto: Fernando Istaña 21 · Henry Ticona 63 · Nicolás Pachamora 31 · Víctor Luján 38</t>
         </is>
       </c>
       <c r="C43" s="2" t="n"/>
@@ -2834,7 +2834,7 @@
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
@@ -2920,7 +2920,7 @@
     <row r="81" ht="18" customHeight="1">
       <c r="B81" s="18" t="inlineStr">
         <is>
-          <t>Total: 107 puntos en 31 historias.  Reparto: Fernando Istaña 5 · Henry Ticona 48 · Nicolás Pachamora 24 · Víctor Luján 30</t>
+          <t>Total: 108 puntos en 31 historias.  Reparto: Fernando Istaña 5 · Henry Ticona 49 · Nicolás Pachamora 24 · Víctor Luján 30</t>
         </is>
       </c>
       <c r="C81" s="2" t="n"/>
@@ -3072,7 +3072,7 @@
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G87" s="12" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="F88" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G88" s="16" t="inlineStr">
         <is>

</xml_diff>